<commit_message>
Add final RMS quotes (RFQ 27, requisitions 30/31)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FAbqBnpuWH1yd5Twkz2bzr
</commit_message>
<xml_diff>
--- a/선박별_견적관리.xlsx
+++ b/선박별_견적관리.xlsx
@@ -12715,24 +12715,70 @@
         <f>IF(E19="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B19" s="36" t="n"/>
-      <c r="C19" s="36" t="n"/>
-      <c r="D19" s="36" t="n"/>
-      <c r="E19" s="37" t="n"/>
-      <c r="F19" s="37" t="n"/>
+      <c r="B19" s="36" t="inlineStr">
+        <is>
+          <t>KQU-000116301</t>
+        </is>
+      </c>
+      <c r="C19" s="36" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D19" s="36" t="inlineStr">
+        <is>
+          <t>MRC</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="inlineStr">
+        <is>
+          <t>Handset with cord</t>
+        </is>
+      </c>
+      <c r="F19" s="37" t="inlineStr">
+        <is>
+          <t>MRC / LVD -115D</t>
+        </is>
+      </c>
       <c r="G19" s="37" t="n"/>
-      <c r="H19" s="37" t="n"/>
-      <c r="I19" s="37" t="n"/>
-      <c r="J19" s="36" t="n"/>
-      <c r="K19" s="36" t="n"/>
-      <c r="L19" s="36" t="n"/>
-      <c r="M19" s="36" t="n"/>
-      <c r="N19" s="38" t="n"/>
+      <c r="H19" s="37" t="inlineStr">
+        <is>
+          <t>Telephone system</t>
+        </is>
+      </c>
+      <c r="I19" s="37" t="inlineStr">
+        <is>
+          <t>RMS: 전화기 ASSY로 견적</t>
+        </is>
+      </c>
+      <c r="J19" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="36" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L19" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M19" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N19" s="38" t="n">
+        <v>390000</v>
+      </c>
       <c r="O19" s="39">
         <f>IF(OR(N19="",J19=""),"",N19*J19)</f>
         <v/>
       </c>
-      <c r="P19" s="40" t="n"/>
+      <c r="P19" s="40" t="n">
+        <v>14</v>
+      </c>
       <c r="Q19" s="41">
         <f>IF(OR(P19="",Y19="발주완료",Y19="취소"),"",TODAY()+P19)</f>
         <v/>
@@ -12741,17 +12787,37 @@
         <f>IF(OR(Q19="",NOT(ISNUMBER($J$2))),"",IF(Q19&lt;=$J$2,"가능","초과 "&amp;(Q19-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S19" s="36" t="n"/>
-      <c r="T19" s="36" t="n"/>
+      <c r="S19" s="36" t="inlineStr">
+        <is>
+          <t>COMPATIBLE</t>
+        </is>
+      </c>
+      <c r="T19" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
       <c r="U19" s="36" t="n"/>
-      <c r="V19" s="43" t="n"/>
+      <c r="V19" s="42" t="n"/>
       <c r="W19" s="41">
         <f>IF(OR(V19="",U19=""),"",V19+U19)</f>
         <v/>
       </c>
-      <c r="X19" s="37" t="n"/>
-      <c r="Y19" s="36" t="n"/>
-      <c r="Z19" s="37" t="n"/>
+      <c r="X19" s="37" t="inlineStr">
+        <is>
+          <t>QUOTE AS TELEPHONE ASSY &amp; NEED TO CHECK IP ADDRESS, ID &amp; PASSWORD // D/T: 10 WORKING DAYS, COMPATIBLE, EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="Y19" s="36" t="inlineStr">
+        <is>
+          <t>정보 송부필요</t>
+        </is>
+      </c>
+      <c r="Z19" s="37" t="inlineStr">
+        <is>
+          <t>IP 주소·ID·비밀번호 확인해 RMS 회신 / 호환품(COMPATIBLE) 승인 여부 / 유효기간 미기재</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="35">
@@ -30856,24 +30922,74 @@
         <f>IF(E11="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B11" s="36" t="n"/>
-      <c r="C11" s="36" t="n"/>
-      <c r="D11" s="36" t="n"/>
-      <c r="E11" s="37" t="n"/>
-      <c r="F11" s="37" t="n"/>
-      <c r="G11" s="37" t="n"/>
-      <c r="H11" s="37" t="n"/>
-      <c r="I11" s="37" t="n"/>
-      <c r="J11" s="36" t="n"/>
-      <c r="K11" s="36" t="n"/>
-      <c r="L11" s="36" t="n"/>
-      <c r="M11" s="36" t="n"/>
-      <c r="N11" s="38" t="n"/>
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-30</t>
+        </is>
+      </c>
+      <c r="C11" s="36" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D11" s="36" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>Solenoid Valve for Ballast Hyd. System D1VW4CNJWF (THR TYPE)</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="G11" s="37" t="inlineStr">
+        <is>
+          <t>VPKVVDV4301</t>
+        </is>
+      </c>
+      <c r="H11" s="37" t="inlineStr">
+        <is>
+          <t>Hyd.VRC</t>
+        </is>
+      </c>
+      <c r="I11" s="37" t="inlineStr">
+        <is>
+          <t>DWG:VO61-W2008-9 / RMS: 신형 D1VW004CNJW로 견적</t>
+        </is>
+      </c>
+      <c r="J11" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="36" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L11" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M11" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N11" s="38" t="n">
+        <v>500000</v>
+      </c>
       <c r="O11" s="39">
         <f>IF(OR(N11="",J11=""),"",N11*J11)</f>
         <v/>
       </c>
-      <c r="P11" s="40" t="n"/>
+      <c r="P11" s="40" t="n">
+        <v>90</v>
+      </c>
       <c r="Q11" s="41">
         <f>IF(OR(P11="",Y11="발주완료",Y11="취소"),"",TODAY()+P11)</f>
         <v/>
@@ -30882,41 +30998,113 @@
         <f>IF(OR(Q11="",NOT(ISNUMBER($J$2))),"",IF(Q11&lt;=$J$2,"가능","초과 "&amp;(Q11-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S11" s="36" t="n"/>
-      <c r="T11" s="36" t="n"/>
-      <c r="U11" s="36" t="n"/>
-      <c r="V11" s="43" t="n"/>
+      <c r="S11" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T11" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U11" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V11" s="42" t="n"/>
       <c r="W11" s="41">
         <f>IF(OR(V11="",U11=""),"",V11+U11)</f>
         <v/>
       </c>
-      <c r="X11" s="37" t="n"/>
-      <c r="Y11" s="36" t="n"/>
-      <c r="Z11" s="37" t="n"/>
+      <c r="X11" s="37" t="inlineStr">
+        <is>
+          <t>#1 = QUOTE AS NEW TYPE: D1VW004CNJW (OBSOLETE D1VW4CNJWF) / D/T: 90 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y11" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
+      <c r="Z11" s="37" t="inlineStr">
+        <is>
+          <t>신형 대체품 호환 확인</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="35">
         <f>IF(E12="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B12" s="36" t="n"/>
-      <c r="C12" s="36" t="n"/>
-      <c r="D12" s="36" t="n"/>
-      <c r="E12" s="37" t="n"/>
-      <c r="F12" s="37" t="n"/>
-      <c r="G12" s="37" t="n"/>
-      <c r="H12" s="37" t="n"/>
-      <c r="I12" s="37" t="n"/>
-      <c r="J12" s="36" t="n"/>
-      <c r="K12" s="36" t="n"/>
-      <c r="L12" s="36" t="n"/>
-      <c r="M12" s="36" t="n"/>
-      <c r="N12" s="38" t="n"/>
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-30</t>
+        </is>
+      </c>
+      <c r="C12" s="36" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D12" s="36" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>Solenoid Valve for Ballast Hyd. System D1VW20DNJWF (O/S TYPE)</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>Parker</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
+        <is>
+          <t>VPKVVDV4201</t>
+        </is>
+      </c>
+      <c r="H12" s="37" t="inlineStr">
+        <is>
+          <t>Hyd.VRC</t>
+        </is>
+      </c>
+      <c r="I12" s="37" t="inlineStr">
+        <is>
+          <t>DWG:VO61-W2008-10 / RMS: 신형 D1VW020DNJW로 견적</t>
+        </is>
+      </c>
+      <c r="J12" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="36" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L12" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M12" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N12" s="38" t="n">
+        <v>649000</v>
+      </c>
       <c r="O12" s="39">
         <f>IF(OR(N12="",J12=""),"",N12*J12)</f>
         <v/>
       </c>
-      <c r="P12" s="40" t="n"/>
+      <c r="P12" s="40" t="n">
+        <v>90</v>
+      </c>
       <c r="Q12" s="41">
         <f>IF(OR(P12="",Y12="발주완료",Y12="취소"),"",TODAY()+P12)</f>
         <v/>
@@ -30925,35 +31113,95 @@
         <f>IF(OR(Q12="",NOT(ISNUMBER($J$2))),"",IF(Q12&lt;=$J$2,"가능","초과 "&amp;(Q12-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S12" s="36" t="n"/>
-      <c r="T12" s="36" t="n"/>
-      <c r="U12" s="36" t="n"/>
-      <c r="V12" s="43" t="n"/>
+      <c r="S12" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U12" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V12" s="42" t="n"/>
       <c r="W12" s="41">
         <f>IF(OR(V12="",U12=""),"",V12+U12)</f>
         <v/>
       </c>
-      <c r="X12" s="37" t="n"/>
-      <c r="Y12" s="36" t="n"/>
-      <c r="Z12" s="37" t="n"/>
+      <c r="X12" s="37" t="inlineStr">
+        <is>
+          <t>#2 = QUOTE AS NEW TYPE: D1VW020DNJW (OBSOLETE D1VW020DNJW) / D/T: 90 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y12" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
+      <c r="Z12" s="37" t="inlineStr">
+        <is>
+          <t>신형 대체품 호환 확인 (RMS 비고의 OBSOLETE 형번 오기 확인)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="35">
         <f>IF(E13="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B13" s="36" t="n"/>
-      <c r="C13" s="36" t="n"/>
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-30</t>
+        </is>
+      </c>
+      <c r="C13" s="36" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="D13" s="36" t="n"/>
-      <c r="E13" s="37" t="n"/>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>Solenoid Valve for Ballast Hyd. System DHW-0713P</t>
+        </is>
+      </c>
       <c r="F13" s="37" t="n"/>
-      <c r="G13" s="37" t="n"/>
-      <c r="H13" s="37" t="n"/>
-      <c r="I13" s="37" t="n"/>
-      <c r="J13" s="36" t="n"/>
-      <c r="K13" s="36" t="n"/>
-      <c r="L13" s="36" t="n"/>
-      <c r="M13" s="36" t="n"/>
+      <c r="G13" s="37" t="inlineStr">
+        <is>
+          <t>VATVDV43001</t>
+        </is>
+      </c>
+      <c r="H13" s="37" t="inlineStr">
+        <is>
+          <t>Hyd.VRC</t>
+        </is>
+      </c>
+      <c r="I13" s="37" t="inlineStr">
+        <is>
+          <t>DWG:VO61-W2008-6</t>
+        </is>
+      </c>
+      <c r="J13" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="36" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L13" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M13" s="36" t="inlineStr">
+        <is>
+          <t>공급불가</t>
+        </is>
+      </c>
       <c r="N13" s="38" t="n"/>
       <c r="O13" s="39">
         <f>IF(OR(N13="",J13=""),"",N13*J13)</f>
@@ -30971,32 +31219,82 @@
       <c r="S13" s="36" t="n"/>
       <c r="T13" s="36" t="n"/>
       <c r="U13" s="36" t="n"/>
-      <c r="V13" s="43" t="n"/>
+      <c r="V13" s="42" t="n"/>
       <c r="W13" s="41">
         <f>IF(OR(V13="",U13=""),"",V13+U13)</f>
         <v/>
       </c>
-      <c r="X13" s="37" t="n"/>
-      <c r="Y13" s="36" t="n"/>
-      <c r="Z13" s="37" t="n"/>
+      <c r="X13" s="37" t="inlineStr">
+        <is>
+          <t>NOT AVAILABLE</t>
+        </is>
+      </c>
+      <c r="Y13" s="36" t="inlineStr">
+        <is>
+          <t>타업체 문의</t>
+        </is>
+      </c>
+      <c r="Z13" s="37" t="inlineStr">
+        <is>
+          <t>타 업체 견적 요청</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="35">
         <f>IF(E14="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B14" s="36" t="n"/>
-      <c r="C14" s="36" t="n"/>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-30</t>
+        </is>
+      </c>
+      <c r="C14" s="36" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="D14" s="36" t="n"/>
-      <c r="E14" s="37" t="n"/>
+      <c r="E14" s="37" t="inlineStr">
+        <is>
+          <t>Solenoid Valve for Ballast Hyd. System DHW-0751/2</t>
+        </is>
+      </c>
       <c r="F14" s="37" t="n"/>
-      <c r="G14" s="37" t="n"/>
-      <c r="H14" s="37" t="n"/>
-      <c r="I14" s="37" t="n"/>
-      <c r="J14" s="36" t="n"/>
-      <c r="K14" s="36" t="n"/>
-      <c r="L14" s="36" t="n"/>
-      <c r="M14" s="36" t="n"/>
+      <c r="G14" s="37" t="inlineStr">
+        <is>
+          <t>VATVDV42005</t>
+        </is>
+      </c>
+      <c r="H14" s="37" t="inlineStr">
+        <is>
+          <t>Hyd.VRC</t>
+        </is>
+      </c>
+      <c r="I14" s="37" t="inlineStr">
+        <is>
+          <t>DWG:VO61-W2008-7</t>
+        </is>
+      </c>
+      <c r="J14" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="36" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L14" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M14" s="36" t="inlineStr">
+        <is>
+          <t>공급불가</t>
+        </is>
+      </c>
       <c r="N14" s="38" t="n"/>
       <c r="O14" s="39">
         <f>IF(OR(N14="",J14=""),"",N14*J14)</f>
@@ -31014,38 +31312,96 @@
       <c r="S14" s="36" t="n"/>
       <c r="T14" s="36" t="n"/>
       <c r="U14" s="36" t="n"/>
-      <c r="V14" s="43" t="n"/>
+      <c r="V14" s="42" t="n"/>
       <c r="W14" s="41">
         <f>IF(OR(V14="",U14=""),"",V14+U14)</f>
         <v/>
       </c>
-      <c r="X14" s="37" t="n"/>
-      <c r="Y14" s="36" t="n"/>
-      <c r="Z14" s="37" t="n"/>
+      <c r="X14" s="37" t="inlineStr">
+        <is>
+          <t>NOT AVAILABLE</t>
+        </is>
+      </c>
+      <c r="Y14" s="36" t="inlineStr">
+        <is>
+          <t>타업체 문의</t>
+        </is>
+      </c>
+      <c r="Z14" s="37" t="inlineStr">
+        <is>
+          <t>타 업체 견적 요청</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="35">
         <f>IF(E15="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B15" s="36" t="n"/>
-      <c r="C15" s="36" t="n"/>
-      <c r="D15" s="36" t="n"/>
-      <c r="E15" s="37" t="n"/>
-      <c r="F15" s="37" t="n"/>
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C15" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D15" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E15" s="37" t="inlineStr">
+        <is>
+          <t>PUMP COMPLETE</t>
+        </is>
+      </c>
+      <c r="F15" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
       <c r="G15" s="37" t="n"/>
-      <c r="H15" s="37" t="n"/>
-      <c r="I15" s="37" t="n"/>
-      <c r="J15" s="36" t="n"/>
-      <c r="K15" s="36" t="n"/>
-      <c r="L15" s="36" t="n"/>
-      <c r="M15" s="36" t="n"/>
-      <c r="N15" s="38" t="n"/>
+      <c r="H15" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
+      <c r="I15" s="37" t="inlineStr">
+        <is>
+          <t>RMS: 모터 포함 펌프 완품으로 견적</t>
+        </is>
+      </c>
+      <c r="J15" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="36" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="L15" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M15" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N15" s="38" t="n">
+        <v>1996560</v>
+      </c>
       <c r="O15" s="39">
         <f>IF(OR(N15="",J15=""),"",N15*J15)</f>
         <v/>
       </c>
-      <c r="P15" s="40" t="n"/>
+      <c r="P15" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q15" s="41">
         <f>IF(OR(P15="",Y15="발주완료",Y15="취소"),"",TODAY()+P15)</f>
         <v/>
@@ -31054,41 +31410,109 @@
         <f>IF(OR(Q15="",NOT(ISNUMBER($J$2))),"",IF(Q15&lt;=$J$2,"가능","초과 "&amp;(Q15-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S15" s="36" t="n"/>
-      <c r="T15" s="36" t="n"/>
-      <c r="U15" s="36" t="n"/>
-      <c r="V15" s="43" t="n"/>
+      <c r="S15" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T15" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U15" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V15" s="42" t="n"/>
       <c r="W15" s="41">
         <f>IF(OR(V15="",U15=""),"",V15+U15)</f>
         <v/>
       </c>
-      <c r="X15" s="37" t="n"/>
-      <c r="Y15" s="36" t="n"/>
-      <c r="Z15" s="37" t="n"/>
+      <c r="X15" s="37" t="inlineStr">
+        <is>
+          <t>#1 = QUOTE AS PUMP WITH MOTOR COMPLETE (→ Motor Rated voltage : 3 x 220-255D / 380-440Y V, 60HZ에 사용 됩니다. / ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y15" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
+      <c r="Z15" s="37" t="inlineStr">
+        <is>
+          <t>모터 전압/60Hz 선내 사양 일치 확인</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="35">
         <f>IF(E16="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B16" s="36" t="n"/>
-      <c r="C16" s="36" t="n"/>
-      <c r="D16" s="36" t="n"/>
-      <c r="E16" s="37" t="n"/>
-      <c r="F16" s="37" t="n"/>
-      <c r="G16" s="37" t="n"/>
-      <c r="H16" s="37" t="n"/>
+      <c r="B16" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D16" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E16" s="37" t="inlineStr">
+        <is>
+          <t>O-RING</t>
+        </is>
+      </c>
+      <c r="F16" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G16" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-37</t>
+        </is>
+      </c>
+      <c r="H16" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I16" s="37" t="n"/>
-      <c r="J16" s="36" t="n"/>
-      <c r="K16" s="36" t="n"/>
-      <c r="L16" s="36" t="n"/>
-      <c r="M16" s="36" t="n"/>
-      <c r="N16" s="38" t="n"/>
+      <c r="J16" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L16" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M16" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N16" s="38" t="n">
+        <v>16638</v>
+      </c>
       <c r="O16" s="39">
         <f>IF(OR(N16="",J16=""),"",N16*J16)</f>
         <v/>
       </c>
-      <c r="P16" s="40" t="n"/>
+      <c r="P16" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q16" s="41">
         <f>IF(OR(P16="",Y16="발주완료",Y16="취소"),"",TODAY()+P16)</f>
         <v/>
@@ -31097,16 +31521,34 @@
         <f>IF(OR(Q16="",NOT(ISNUMBER($J$2))),"",IF(Q16&lt;=$J$2,"가능","초과 "&amp;(Q16-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S16" s="36" t="n"/>
-      <c r="T16" s="36" t="n"/>
-      <c r="U16" s="36" t="n"/>
-      <c r="V16" s="43" t="n"/>
+      <c r="S16" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T16" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U16" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V16" s="42" t="n"/>
       <c r="W16" s="41">
         <f>IF(OR(V16="",U16=""),"",V16+U16)</f>
         <v/>
       </c>
-      <c r="X16" s="37" t="n"/>
-      <c r="Y16" s="36" t="n"/>
+      <c r="X16" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y16" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z16" s="37" t="n"/>
     </row>
     <row r="17">
@@ -31114,24 +31556,70 @@
         <f>IF(E17="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B17" s="36" t="n"/>
-      <c r="C17" s="36" t="n"/>
-      <c r="D17" s="36" t="n"/>
-      <c r="E17" s="37" t="n"/>
-      <c r="F17" s="37" t="n"/>
-      <c r="G17" s="37" t="n"/>
-      <c r="H17" s="37" t="n"/>
+      <c r="B17" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D17" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E17" s="37" t="inlineStr">
+        <is>
+          <t>CHAMBER</t>
+        </is>
+      </c>
+      <c r="F17" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G17" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-4</t>
+        </is>
+      </c>
+      <c r="H17" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I17" s="37" t="n"/>
-      <c r="J17" s="36" t="n"/>
-      <c r="K17" s="36" t="n"/>
-      <c r="L17" s="36" t="n"/>
-      <c r="M17" s="36" t="n"/>
-      <c r="N17" s="38" t="n"/>
+      <c r="J17" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="K17" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L17" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M17" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N17" s="38" t="n">
+        <v>44368</v>
+      </c>
       <c r="O17" s="39">
         <f>IF(OR(N17="",J17=""),"",N17*J17)</f>
         <v/>
       </c>
-      <c r="P17" s="40" t="n"/>
+      <c r="P17" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q17" s="41">
         <f>IF(OR(P17="",Y17="발주완료",Y17="취소"),"",TODAY()+P17)</f>
         <v/>
@@ -31140,16 +31628,34 @@
         <f>IF(OR(Q17="",NOT(ISNUMBER($J$2))),"",IF(Q17&lt;=$J$2,"가능","초과 "&amp;(Q17-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S17" s="36" t="n"/>
-      <c r="T17" s="36" t="n"/>
-      <c r="U17" s="36" t="n"/>
-      <c r="V17" s="43" t="n"/>
+      <c r="S17" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T17" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U17" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V17" s="42" t="n"/>
       <c r="W17" s="41">
         <f>IF(OR(V17="",U17=""),"",V17+U17)</f>
         <v/>
       </c>
-      <c r="X17" s="37" t="n"/>
-      <c r="Y17" s="36" t="n"/>
+      <c r="X17" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y17" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z17" s="37" t="n"/>
     </row>
     <row r="18">
@@ -31157,24 +31663,70 @@
         <f>IF(E18="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B18" s="36" t="n"/>
-      <c r="C18" s="36" t="n"/>
-      <c r="D18" s="36" t="n"/>
-      <c r="E18" s="37" t="n"/>
-      <c r="F18" s="37" t="n"/>
-      <c r="G18" s="37" t="n"/>
-      <c r="H18" s="37" t="n"/>
+      <c r="B18" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C18" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D18" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E18" s="37" t="inlineStr">
+        <is>
+          <t>CHAMBER WITH BEARING</t>
+        </is>
+      </c>
+      <c r="F18" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G18" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-4A</t>
+        </is>
+      </c>
+      <c r="H18" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I18" s="37" t="n"/>
-      <c r="J18" s="36" t="n"/>
-      <c r="K18" s="36" t="n"/>
-      <c r="L18" s="36" t="n"/>
-      <c r="M18" s="36" t="n"/>
-      <c r="N18" s="38" t="n"/>
+      <c r="J18" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L18" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M18" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N18" s="38" t="n">
+        <v>49914</v>
+      </c>
       <c r="O18" s="39">
         <f>IF(OR(N18="",J18=""),"",N18*J18)</f>
         <v/>
       </c>
-      <c r="P18" s="40" t="n"/>
+      <c r="P18" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q18" s="41">
         <f>IF(OR(P18="",Y18="발주완료",Y18="취소"),"",TODAY()+P18)</f>
         <v/>
@@ -31183,16 +31735,34 @@
         <f>IF(OR(Q18="",NOT(ISNUMBER($J$2))),"",IF(Q18&lt;=$J$2,"가능","초과 "&amp;(Q18-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S18" s="36" t="n"/>
-      <c r="T18" s="36" t="n"/>
-      <c r="U18" s="36" t="n"/>
-      <c r="V18" s="43" t="n"/>
+      <c r="S18" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T18" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U18" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V18" s="42" t="n"/>
       <c r="W18" s="41">
         <f>IF(OR(V18="",U18=""),"",V18+U18)</f>
         <v/>
       </c>
-      <c r="X18" s="37" t="n"/>
-      <c r="Y18" s="36" t="n"/>
+      <c r="X18" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y18" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z18" s="37" t="n"/>
     </row>
     <row r="19">
@@ -31200,24 +31770,70 @@
         <f>IF(E19="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B19" s="36" t="n"/>
-      <c r="C19" s="36" t="n"/>
-      <c r="D19" s="36" t="n"/>
-      <c r="E19" s="37" t="n"/>
-      <c r="F19" s="37" t="n"/>
-      <c r="G19" s="37" t="n"/>
-      <c r="H19" s="37" t="n"/>
+      <c r="B19" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C19" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D19" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="inlineStr">
+        <is>
+          <t>SPACING PIPE</t>
+        </is>
+      </c>
+      <c r="F19" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G19" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-64</t>
+        </is>
+      </c>
+      <c r="H19" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I19" s="37" t="n"/>
-      <c r="J19" s="36" t="n"/>
-      <c r="K19" s="36" t="n"/>
-      <c r="L19" s="36" t="n"/>
-      <c r="M19" s="36" t="n"/>
-      <c r="N19" s="38" t="n"/>
+      <c r="J19" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="K19" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L19" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M19" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N19" s="38" t="n">
+        <v>9982.799999999999</v>
+      </c>
       <c r="O19" s="39">
         <f>IF(OR(N19="",J19=""),"",N19*J19)</f>
         <v/>
       </c>
-      <c r="P19" s="40" t="n"/>
+      <c r="P19" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q19" s="41">
         <f>IF(OR(P19="",Y19="발주완료",Y19="취소"),"",TODAY()+P19)</f>
         <v/>
@@ -31226,16 +31842,34 @@
         <f>IF(OR(Q19="",NOT(ISNUMBER($J$2))),"",IF(Q19&lt;=$J$2,"가능","초과 "&amp;(Q19-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S19" s="36" t="n"/>
-      <c r="T19" s="36" t="n"/>
-      <c r="U19" s="36" t="n"/>
-      <c r="V19" s="43" t="n"/>
+      <c r="S19" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T19" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U19" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V19" s="42" t="n"/>
       <c r="W19" s="41">
         <f>IF(OR(V19="",U19=""),"",V19+U19)</f>
         <v/>
       </c>
-      <c r="X19" s="37" t="n"/>
-      <c r="Y19" s="36" t="n"/>
+      <c r="X19" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y19" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z19" s="37" t="n"/>
     </row>
     <row r="20">
@@ -31243,24 +31877,70 @@
         <f>IF(E20="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B20" s="36" t="n"/>
-      <c r="C20" s="36" t="n"/>
-      <c r="D20" s="36" t="n"/>
-      <c r="E20" s="37" t="n"/>
-      <c r="F20" s="37" t="n"/>
-      <c r="G20" s="37" t="n"/>
-      <c r="H20" s="37" t="n"/>
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C20" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D20" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E20" s="37" t="inlineStr">
+        <is>
+          <t>SPACING PIPE</t>
+        </is>
+      </c>
+      <c r="F20" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G20" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-64A</t>
+        </is>
+      </c>
+      <c r="H20" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I20" s="37" t="n"/>
-      <c r="J20" s="36" t="n"/>
-      <c r="K20" s="36" t="n"/>
-      <c r="L20" s="36" t="n"/>
-      <c r="M20" s="36" t="n"/>
-      <c r="N20" s="38" t="n"/>
+      <c r="J20" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L20" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M20" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N20" s="38" t="n">
+        <v>6655.2</v>
+      </c>
       <c r="O20" s="39">
         <f>IF(OR(N20="",J20=""),"",N20*J20)</f>
         <v/>
       </c>
-      <c r="P20" s="40" t="n"/>
+      <c r="P20" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q20" s="41">
         <f>IF(OR(P20="",Y20="발주완료",Y20="취소"),"",TODAY()+P20)</f>
         <v/>
@@ -31269,16 +31949,34 @@
         <f>IF(OR(Q20="",NOT(ISNUMBER($J$2))),"",IF(Q20&lt;=$J$2,"가능","초과 "&amp;(Q20-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S20" s="36" t="n"/>
-      <c r="T20" s="36" t="n"/>
-      <c r="U20" s="36" t="n"/>
-      <c r="V20" s="43" t="n"/>
+      <c r="S20" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T20" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U20" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V20" s="42" t="n"/>
       <c r="W20" s="41">
         <f>IF(OR(V20="",U20=""),"",V20+U20)</f>
         <v/>
       </c>
-      <c r="X20" s="37" t="n"/>
-      <c r="Y20" s="36" t="n"/>
+      <c r="X20" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y20" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z20" s="37" t="n"/>
     </row>
     <row r="21">
@@ -31286,24 +31984,70 @@
         <f>IF(E21="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B21" s="36" t="n"/>
-      <c r="C21" s="36" t="n"/>
-      <c r="D21" s="36" t="n"/>
-      <c r="E21" s="37" t="n"/>
-      <c r="F21" s="37" t="n"/>
-      <c r="G21" s="37" t="n"/>
-      <c r="H21" s="37" t="n"/>
+      <c r="B21" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C21" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D21" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E21" s="37" t="inlineStr">
+        <is>
+          <t>SPACING PIPE</t>
+        </is>
+      </c>
+      <c r="F21" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G21" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-64C</t>
+        </is>
+      </c>
+      <c r="H21" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I21" s="37" t="n"/>
-      <c r="J21" s="36" t="n"/>
-      <c r="K21" s="36" t="n"/>
-      <c r="L21" s="36" t="n"/>
-      <c r="M21" s="36" t="n"/>
-      <c r="N21" s="38" t="n"/>
+      <c r="J21" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L21" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M21" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N21" s="38" t="n">
+        <v>27730</v>
+      </c>
       <c r="O21" s="39">
         <f>IF(OR(N21="",J21=""),"",N21*J21)</f>
         <v/>
       </c>
-      <c r="P21" s="40" t="n"/>
+      <c r="P21" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q21" s="41">
         <f>IF(OR(P21="",Y21="발주완료",Y21="취소"),"",TODAY()+P21)</f>
         <v/>
@@ -31312,16 +32056,34 @@
         <f>IF(OR(Q21="",NOT(ISNUMBER($J$2))),"",IF(Q21&lt;=$J$2,"가능","초과 "&amp;(Q21-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S21" s="36" t="n"/>
-      <c r="T21" s="36" t="n"/>
-      <c r="U21" s="36" t="n"/>
-      <c r="V21" s="43" t="n"/>
+      <c r="S21" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T21" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U21" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V21" s="42" t="n"/>
       <c r="W21" s="41">
         <f>IF(OR(V21="",U21=""),"",V21+U21)</f>
         <v/>
       </c>
-      <c r="X21" s="37" t="n"/>
-      <c r="Y21" s="36" t="n"/>
+      <c r="X21" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y21" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z21" s="37" t="n"/>
     </row>
     <row r="22">
@@ -31329,18 +32091,56 @@
         <f>IF(E22="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B22" s="36" t="n"/>
-      <c r="C22" s="36" t="n"/>
-      <c r="D22" s="36" t="n"/>
-      <c r="E22" s="37" t="n"/>
-      <c r="F22" s="37" t="n"/>
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C22" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D22" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E22" s="37" t="inlineStr">
+        <is>
+          <t>PACKING FOR IMPELLER</t>
+        </is>
+      </c>
+      <c r="F22" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-8</t>
+        </is>
+      </c>
       <c r="G22" s="37" t="n"/>
-      <c r="H22" s="37" t="n"/>
+      <c r="H22" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I22" s="37" t="n"/>
-      <c r="J22" s="36" t="n"/>
-      <c r="K22" s="36" t="n"/>
-      <c r="L22" s="36" t="n"/>
-      <c r="M22" s="36" t="n"/>
+      <c r="J22" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="K22" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L22" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M22" s="36" t="inlineStr">
+        <is>
+          <t>공급불가</t>
+        </is>
+      </c>
       <c r="N22" s="38" t="n"/>
       <c r="O22" s="39">
         <f>IF(OR(N22="",J22=""),"",N22*J22)</f>
@@ -31358,38 +32158,96 @@
       <c r="S22" s="36" t="n"/>
       <c r="T22" s="36" t="n"/>
       <c r="U22" s="36" t="n"/>
-      <c r="V22" s="43" t="n"/>
+      <c r="V22" s="42" t="n"/>
       <c r="W22" s="41">
         <f>IF(OR(V22="",U22=""),"",V22+U22)</f>
         <v/>
       </c>
-      <c r="X22" s="37" t="n"/>
-      <c r="Y22" s="36" t="n"/>
-      <c r="Z22" s="37" t="n"/>
+      <c r="X22" s="37" t="inlineStr">
+        <is>
+          <t>NOT AVAILABLE</t>
+        </is>
+      </c>
+      <c r="Y22" s="36" t="inlineStr">
+        <is>
+          <t>타업체 문의</t>
+        </is>
+      </c>
+      <c r="Z22" s="37" t="inlineStr">
+        <is>
+          <t>타 업체 견적 요청</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="35">
         <f>IF(E23="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B23" s="36" t="n"/>
-      <c r="C23" s="36" t="n"/>
-      <c r="D23" s="36" t="n"/>
-      <c r="E23" s="37" t="n"/>
-      <c r="F23" s="37" t="n"/>
-      <c r="G23" s="37" t="n"/>
-      <c r="H23" s="37" t="n"/>
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C23" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D23" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E23" s="37" t="inlineStr">
+        <is>
+          <t>IMPELLER</t>
+        </is>
+      </c>
+      <c r="F23" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G23" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-49</t>
+        </is>
+      </c>
+      <c r="H23" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I23" s="37" t="n"/>
-      <c r="J23" s="36" t="n"/>
-      <c r="K23" s="36" t="n"/>
-      <c r="L23" s="36" t="n"/>
-      <c r="M23" s="36" t="n"/>
-      <c r="N23" s="38" t="n"/>
+      <c r="J23" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="K23" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L23" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M23" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N23" s="38" t="n">
+        <v>33276</v>
+      </c>
       <c r="O23" s="39">
         <f>IF(OR(N23="",J23=""),"",N23*J23)</f>
         <v/>
       </c>
-      <c r="P23" s="40" t="n"/>
+      <c r="P23" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q23" s="41">
         <f>IF(OR(P23="",Y23="발주완료",Y23="취소"),"",TODAY()+P23)</f>
         <v/>
@@ -31398,16 +32256,34 @@
         <f>IF(OR(Q23="",NOT(ISNUMBER($J$2))),"",IF(Q23&lt;=$J$2,"가능","초과 "&amp;(Q23-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S23" s="36" t="n"/>
-      <c r="T23" s="36" t="n"/>
-      <c r="U23" s="36" t="n"/>
-      <c r="V23" s="43" t="n"/>
+      <c r="S23" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T23" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U23" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V23" s="42" t="n"/>
       <c r="W23" s="41">
         <f>IF(OR(V23="",U23=""),"",V23+U23)</f>
         <v/>
       </c>
-      <c r="X23" s="37" t="n"/>
-      <c r="Y23" s="36" t="n"/>
+      <c r="X23" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y23" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z23" s="37" t="n"/>
     </row>
     <row r="24">
@@ -31415,18 +32291,60 @@
         <f>IF(E24="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B24" s="36" t="n"/>
-      <c r="C24" s="36" t="n"/>
-      <c r="D24" s="36" t="n"/>
-      <c r="E24" s="37" t="n"/>
-      <c r="F24" s="37" t="n"/>
-      <c r="G24" s="37" t="n"/>
-      <c r="H24" s="37" t="n"/>
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C24" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D24" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E24" s="37" t="inlineStr">
+        <is>
+          <t>IMPELLER, SPECIAL</t>
+        </is>
+      </c>
+      <c r="F24" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G24" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-49G</t>
+        </is>
+      </c>
+      <c r="H24" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I24" s="37" t="n"/>
-      <c r="J24" s="36" t="n"/>
-      <c r="K24" s="36" t="n"/>
-      <c r="L24" s="36" t="n"/>
-      <c r="M24" s="36" t="n"/>
+      <c r="J24" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L24" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M24" s="36" t="inlineStr">
+        <is>
+          <t>공급불가</t>
+        </is>
+      </c>
       <c r="N24" s="38" t="n"/>
       <c r="O24" s="39">
         <f>IF(OR(N24="",J24=""),"",N24*J24)</f>
@@ -31444,38 +32362,96 @@
       <c r="S24" s="36" t="n"/>
       <c r="T24" s="36" t="n"/>
       <c r="U24" s="36" t="n"/>
-      <c r="V24" s="43" t="n"/>
+      <c r="V24" s="42" t="n"/>
       <c r="W24" s="41">
         <f>IF(OR(V24="",U24=""),"",V24+U24)</f>
         <v/>
       </c>
-      <c r="X24" s="37" t="n"/>
-      <c r="Y24" s="36" t="n"/>
-      <c r="Z24" s="37" t="n"/>
+      <c r="X24" s="37" t="inlineStr">
+        <is>
+          <t>NOT AVAILABLE</t>
+        </is>
+      </c>
+      <c r="Y24" s="36" t="inlineStr">
+        <is>
+          <t>타업체 문의</t>
+        </is>
+      </c>
+      <c r="Z24" s="37" t="inlineStr">
+        <is>
+          <t>타 업체 견적 요청</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="35">
         <f>IF(E25="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B25" s="36" t="n"/>
-      <c r="C25" s="36" t="n"/>
-      <c r="D25" s="36" t="n"/>
-      <c r="E25" s="37" t="n"/>
-      <c r="F25" s="37" t="n"/>
-      <c r="G25" s="37" t="n"/>
-      <c r="H25" s="37" t="n"/>
+      <c r="B25" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C25" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D25" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E25" s="37" t="inlineStr">
+        <is>
+          <t>WASHER</t>
+        </is>
+      </c>
+      <c r="F25" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G25" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-66</t>
+        </is>
+      </c>
+      <c r="H25" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I25" s="37" t="n"/>
-      <c r="J25" s="36" t="n"/>
-      <c r="K25" s="36" t="n"/>
-      <c r="L25" s="36" t="n"/>
-      <c r="M25" s="36" t="n"/>
-      <c r="N25" s="38" t="n"/>
+      <c r="J25" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="K25" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L25" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M25" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N25" s="38" t="n">
+        <v>14419.6</v>
+      </c>
       <c r="O25" s="39">
         <f>IF(OR(N25="",J25=""),"",N25*J25)</f>
         <v/>
       </c>
-      <c r="P25" s="40" t="n"/>
+      <c r="P25" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q25" s="41">
         <f>IF(OR(P25="",Y25="발주완료",Y25="취소"),"",TODAY()+P25)</f>
         <v/>
@@ -31484,16 +32460,34 @@
         <f>IF(OR(Q25="",NOT(ISNUMBER($J$2))),"",IF(Q25&lt;=$J$2,"가능","초과 "&amp;(Q25-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S25" s="36" t="n"/>
-      <c r="T25" s="36" t="n"/>
-      <c r="U25" s="36" t="n"/>
-      <c r="V25" s="43" t="n"/>
+      <c r="S25" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T25" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U25" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V25" s="42" t="n"/>
       <c r="W25" s="41">
         <f>IF(OR(V25="",U25=""),"",V25+U25)</f>
         <v/>
       </c>
-      <c r="X25" s="37" t="n"/>
-      <c r="Y25" s="36" t="n"/>
+      <c r="X25" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y25" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z25" s="37" t="n"/>
     </row>
     <row r="26">
@@ -31501,24 +32495,70 @@
         <f>IF(E26="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B26" s="36" t="n"/>
-      <c r="C26" s="36" t="n"/>
-      <c r="D26" s="36" t="n"/>
-      <c r="E26" s="37" t="n"/>
-      <c r="F26" s="37" t="n"/>
-      <c r="G26" s="37" t="n"/>
-      <c r="H26" s="37" t="n"/>
+      <c r="B26" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C26" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D26" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E26" s="37" t="inlineStr">
+        <is>
+          <t>NUT</t>
+        </is>
+      </c>
+      <c r="F26" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G26" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-67</t>
+        </is>
+      </c>
+      <c r="H26" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I26" s="37" t="n"/>
-      <c r="J26" s="36" t="n"/>
-      <c r="K26" s="36" t="n"/>
-      <c r="L26" s="36" t="n"/>
-      <c r="M26" s="36" t="n"/>
-      <c r="N26" s="38" t="n"/>
+      <c r="J26" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L26" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M26" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N26" s="38" t="n">
+        <v>8873.6</v>
+      </c>
       <c r="O26" s="39">
         <f>IF(OR(N26="",J26=""),"",N26*J26)</f>
         <v/>
       </c>
-      <c r="P26" s="40" t="n"/>
+      <c r="P26" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q26" s="41">
         <f>IF(OR(P26="",Y26="발주완료",Y26="취소"),"",TODAY()+P26)</f>
         <v/>
@@ -31527,16 +32567,34 @@
         <f>IF(OR(Q26="",NOT(ISNUMBER($J$2))),"",IF(Q26&lt;=$J$2,"가능","초과 "&amp;(Q26-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S26" s="36" t="n"/>
-      <c r="T26" s="36" t="n"/>
-      <c r="U26" s="36" t="n"/>
-      <c r="V26" s="43" t="n"/>
+      <c r="S26" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T26" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U26" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V26" s="42" t="n"/>
       <c r="W26" s="41">
         <f>IF(OR(V26="",U26=""),"",V26+U26)</f>
         <v/>
       </c>
-      <c r="X26" s="37" t="n"/>
-      <c r="Y26" s="36" t="n"/>
+      <c r="X26" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y26" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z26" s="37" t="n"/>
     </row>
     <row r="27">
@@ -31544,24 +32602,66 @@
         <f>IF(E27="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B27" s="36" t="n"/>
-      <c r="C27" s="36" t="n"/>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="37" t="n"/>
-      <c r="F27" s="37" t="n"/>
+      <c r="B27" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C27" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D27" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E27" s="37" t="inlineStr">
+        <is>
+          <t>M/SEAL</t>
+        </is>
+      </c>
+      <c r="F27" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
       <c r="G27" s="37" t="n"/>
-      <c r="H27" s="37" t="n"/>
+      <c r="H27" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I27" s="37" t="n"/>
-      <c r="J27" s="36" t="n"/>
-      <c r="K27" s="36" t="n"/>
-      <c r="L27" s="36" t="n"/>
-      <c r="M27" s="36" t="n"/>
-      <c r="N27" s="38" t="n"/>
+      <c r="J27" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K27" s="36" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="L27" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M27" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N27" s="38" t="n">
+        <v>288392</v>
+      </c>
       <c r="O27" s="39">
         <f>IF(OR(N27="",J27=""),"",N27*J27)</f>
         <v/>
       </c>
-      <c r="P27" s="40" t="n"/>
+      <c r="P27" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q27" s="41">
         <f>IF(OR(P27="",Y27="발주완료",Y27="취소"),"",TODAY()+P27)</f>
         <v/>
@@ -31570,16 +32670,34 @@
         <f>IF(OR(Q27="",NOT(ISNUMBER($J$2))),"",IF(Q27&lt;=$J$2,"가능","초과 "&amp;(Q27-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S27" s="36" t="n"/>
-      <c r="T27" s="36" t="n"/>
-      <c r="U27" s="36" t="n"/>
-      <c r="V27" s="43" t="n"/>
+      <c r="S27" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T27" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U27" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V27" s="42" t="n"/>
       <c r="W27" s="41">
         <f>IF(OR(V27="",U27=""),"",V27+U27)</f>
         <v/>
       </c>
-      <c r="X27" s="37" t="n"/>
-      <c r="Y27" s="36" t="n"/>
+      <c r="X27" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y27" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z27" s="37" t="n"/>
     </row>
     <row r="28">
@@ -31587,24 +32705,70 @@
         <f>IF(E28="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B28" s="36" t="n"/>
-      <c r="C28" s="36" t="n"/>
-      <c r="D28" s="36" t="n"/>
-      <c r="E28" s="37" t="n"/>
-      <c r="F28" s="37" t="n"/>
-      <c r="G28" s="37" t="n"/>
-      <c r="H28" s="37" t="n"/>
+      <c r="B28" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C28" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D28" s="36" t="inlineStr">
+        <is>
+          <t>GRUNDFOS</t>
+        </is>
+      </c>
+      <c r="E28" s="37" t="inlineStr">
+        <is>
+          <t>BEARING RING</t>
+        </is>
+      </c>
+      <c r="F28" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS/CRN3-7</t>
+        </is>
+      </c>
+      <c r="G28" s="37" t="inlineStr">
+        <is>
+          <t>CRN3-7-47A</t>
+        </is>
+      </c>
+      <c r="H28" s="37" t="inlineStr">
+        <is>
+          <t>ME EGR WTS PUMP</t>
+        </is>
+      </c>
       <c r="I28" s="37" t="n"/>
-      <c r="J28" s="36" t="n"/>
-      <c r="K28" s="36" t="n"/>
-      <c r="L28" s="36" t="n"/>
-      <c r="M28" s="36" t="n"/>
-      <c r="N28" s="38" t="n"/>
+      <c r="J28" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="36" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="L28" s="36" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
+      </c>
+      <c r="M28" s="36" t="inlineStr">
+        <is>
+          <t>견적접수</t>
+        </is>
+      </c>
+      <c r="N28" s="38" t="n">
+        <v>33276</v>
+      </c>
       <c r="O28" s="39">
         <f>IF(OR(N28="",J28=""),"",N28*J28)</f>
         <v/>
       </c>
-      <c r="P28" s="40" t="n"/>
+      <c r="P28" s="40" t="n">
+        <v>10</v>
+      </c>
       <c r="Q28" s="41">
         <f>IF(OR(P28="",Y28="발주완료",Y28="취소"),"",TODAY()+P28)</f>
         <v/>
@@ -31613,16 +32777,34 @@
         <f>IF(OR(Q28="",NOT(ISNUMBER($J$2))),"",IF(Q28&lt;=$J$2,"가능","초과 "&amp;(Q28-$J$2)&amp;"일"))</f>
         <v/>
       </c>
-      <c r="S28" s="36" t="n"/>
-      <c r="T28" s="36" t="n"/>
-      <c r="U28" s="36" t="n"/>
-      <c r="V28" s="43" t="n"/>
+      <c r="S28" s="36" t="inlineStr">
+        <is>
+          <t>GENUINE</t>
+        </is>
+      </c>
+      <c r="T28" s="36" t="inlineStr">
+        <is>
+          <t>EX WORK BUSAN</t>
+        </is>
+      </c>
+      <c r="U28" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="V28" s="42" t="n"/>
       <c r="W28" s="41">
         <f>IF(OR(V28="",U28=""),"",V28+U28)</f>
         <v/>
       </c>
-      <c r="X28" s="37" t="n"/>
-      <c r="Y28" s="36" t="n"/>
+      <c r="X28" s="37" t="inlineStr">
+        <is>
+          <t>ALL: D/T: 10 DAYS, GENUINE, EX WORK BUSAN [VALI: 20 DAYS]</t>
+        </is>
+      </c>
+      <c r="Y28" s="36" t="inlineStr">
+        <is>
+          <t>검토중</t>
+        </is>
+      </c>
       <c r="Z28" s="37" t="n"/>
     </row>
     <row r="29">
@@ -39950,13 +41132,37 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="n"/>
-      <c r="B14" s="36" t="n"/>
-      <c r="C14" s="37" t="n"/>
-      <c r="D14" s="36" t="n"/>
-      <c r="E14" s="43" t="n"/>
-      <c r="F14" s="37" t="n"/>
-      <c r="G14" s="36" t="n"/>
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>KQU-000116301</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>MRC (telephone)</t>
+        </is>
+      </c>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>Telephone System</t>
+        </is>
+      </c>
+      <c r="E14" s="43" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F14" s="37" t="inlineStr">
+        <is>
+          <t>MELICERTES</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="n">
+        <v>1</v>
+      </c>
       <c r="H14" s="45">
         <f>IF($B14="","",COUNTIFS('AEOLUS'!$B$6:$B$205,$B14,'AEOLUS'!$M$6:$M$205,"견적접수")+COUNTIFS('MELICERTES'!$B$6:$B$205,$B14,'MELICERTES'!$M$6:$M$205,"견적접수")+COUNTIFS('NELEUS'!$B$6:$B$205,$B14,'NELEUS'!$M$6:$M$205,"견적접수")+COUNTIFS('ONEIROI'!$B$6:$B$205,$B14,'ONEIROI'!$M$6:$M$205,"견적접수"))</f>
         <v/>
@@ -39977,16 +41183,42 @@
         <f>IF($B14="","",SUMIFS('AEOLUS'!$O$6:$O$205,'AEOLUS'!$B$6:$B$205,$B14)+SUMIFS('MELICERTES'!$O$6:$O$205,'MELICERTES'!$B$6:$B$205,$B14)+SUMIFS('NELEUS'!$O$6:$O$205,'NELEUS'!$B$6:$B$205,$B14)+SUMIFS('ONEIROI'!$O$6:$O$205,'ONEIROI'!$B$6:$B$205,$B14))</f>
         <v/>
       </c>
-      <c r="M14" s="37" t="n"/>
+      <c r="M14" s="37" t="inlineStr">
+        <is>
+          <t>RMS 회신</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="36" t="n"/>
-      <c r="B15" s="36" t="n"/>
-      <c r="C15" s="37" t="n"/>
-      <c r="D15" s="36" t="n"/>
+      <c r="A15" s="36" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-30</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>PARKER 외 (Ballast Hyd. solenoid valve)</t>
+        </is>
+      </c>
+      <c r="D15" s="36" t="inlineStr">
+        <is>
+          <t>Hyd. VRC</t>
+        </is>
+      </c>
       <c r="E15" s="43" t="n"/>
-      <c r="F15" s="37" t="n"/>
-      <c r="G15" s="36" t="n"/>
+      <c r="F15" s="37" t="inlineStr">
+        <is>
+          <t>ONEIROI</t>
+        </is>
+      </c>
+      <c r="G15" s="36" t="n">
+        <v>4</v>
+      </c>
       <c r="H15" s="45">
         <f>IF($B15="","",COUNTIFS('AEOLUS'!$B$6:$B$205,$B15,'AEOLUS'!$M$6:$M$205,"견적접수")+COUNTIFS('MELICERTES'!$B$6:$B$205,$B15,'MELICERTES'!$M$6:$M$205,"견적접수")+COUNTIFS('NELEUS'!$B$6:$B$205,$B15,'NELEUS'!$M$6:$M$205,"견적접수")+COUNTIFS('ONEIROI'!$B$6:$B$205,$B15,'ONEIROI'!$M$6:$M$205,"견적접수"))</f>
         <v/>
@@ -40007,16 +41239,44 @@
         <f>IF($B15="","",SUMIFS('AEOLUS'!$O$6:$O$205,'AEOLUS'!$B$6:$B$205,$B15)+SUMIFS('MELICERTES'!$O$6:$O$205,'MELICERTES'!$B$6:$B$205,$B15)+SUMIFS('NELEUS'!$O$6:$O$205,'NELEUS'!$B$6:$B$205,$B15)+SUMIFS('ONEIROI'!$O$6:$O$205,'ONEIROI'!$B$6:$B$205,$B15))</f>
         <v/>
       </c>
-      <c r="M15" s="37" t="n"/>
+      <c r="M15" s="37" t="inlineStr">
+        <is>
+          <t>RMS 회신</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="36" t="n"/>
-      <c r="B16" s="36" t="n"/>
-      <c r="C16" s="37" t="n"/>
-      <c r="D16" s="36" t="n"/>
-      <c r="E16" s="43" t="n"/>
-      <c r="F16" s="37" t="n"/>
-      <c r="G16" s="36" t="n"/>
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="inlineStr">
+        <is>
+          <t>선박요청서-31</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>GRUNDFOS (EGR WTS pump CRN3-7)</t>
+        </is>
+      </c>
+      <c r="D16" s="36" t="inlineStr">
+        <is>
+          <t>Main Engine</t>
+        </is>
+      </c>
+      <c r="E16" s="43" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F16" s="37" t="inlineStr">
+        <is>
+          <t>ONEIROI</t>
+        </is>
+      </c>
+      <c r="G16" s="36" t="n">
+        <v>14</v>
+      </c>
       <c r="H16" s="45">
         <f>IF($B16="","",COUNTIFS('AEOLUS'!$B$6:$B$205,$B16,'AEOLUS'!$M$6:$M$205,"견적접수")+COUNTIFS('MELICERTES'!$B$6:$B$205,$B16,'MELICERTES'!$M$6:$M$205,"견적접수")+COUNTIFS('NELEUS'!$B$6:$B$205,$B16,'NELEUS'!$M$6:$M$205,"견적접수")+COUNTIFS('ONEIROI'!$B$6:$B$205,$B16,'ONEIROI'!$M$6:$M$205,"견적접수"))</f>
         <v/>
@@ -40037,7 +41297,11 @@
         <f>IF($B16="","",SUMIFS('AEOLUS'!$O$6:$O$205,'AEOLUS'!$B$6:$B$205,$B16)+SUMIFS('MELICERTES'!$O$6:$O$205,'MELICERTES'!$B$6:$B$205,$B16)+SUMIFS('NELEUS'!$O$6:$O$205,'NELEUS'!$B$6:$B$205,$B16)+SUMIFS('ONEIROI'!$O$6:$O$205,'ONEIROI'!$B$6:$B$205,$B16))</f>
         <v/>
       </c>
-      <c r="M16" s="37" t="n"/>
+      <c r="M16" s="37" t="inlineStr">
+        <is>
+          <t>RMS 회신</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="36" t="n"/>

</xml_diff>